<commit_message>
updated article brand and zooming
</commit_message>
<xml_diff>
--- a/files/selling_table.xlsx
+++ b/files/selling_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lgc2035/Documents/lawrence-chillrud.github.io/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D24370E-0AAD-B248-8F16-2ECE19D8738C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8544658F-7795-A84F-B275-940E320C0EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{2C9E99C7-C0A1-7B43-AFD4-86135AAC3BC4}"/>
   </bookViews>
@@ -77,9 +77,6 @@
     <t>60x17x27</t>
   </si>
   <si>
-    <t>Bought new in 2022, in mint condition.</t>
-  </si>
-  <si>
     <t>article_stand</t>
   </si>
   <si>
@@ -467,9 +464,6 @@
     <t>utensil_holder</t>
   </si>
   <si>
-    <t>TV stand/console</t>
-  </si>
-  <si>
     <t>Bought in 2024, mint condition. Selling each one for $150, or both for $275.</t>
   </si>
   <si>
@@ -582,6 +576,12 @@
   </si>
   <si>
     <t>Bona Premium Microfiber Floor Mop for Dry and Wet Floor Cleaning - Includes Microfiber Cleaning Pad and Microfiber Dusting Pad</t>
+  </si>
+  <si>
+    <t>Article brand, bought new in 2022, in mint condition.</t>
+  </si>
+  <si>
+    <t>Article TV stand/console</t>
   </si>
 </sst>
 </file>
@@ -1112,7 +1112,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="60">
@@ -1135,12 +1135,12 @@
         <v>10</v>
       </c>
       <c r="H2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="30">
       <c r="A3" s="10" t="s">
-        <v>121</v>
+        <v>159</v>
       </c>
       <c r="B3" s="3">
         <v>849</v>
@@ -1151,22 +1151,22 @@
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="H3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30">
       <c r="A4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" s="3">
         <v>430</v>
@@ -1175,21 +1175,21 @@
         <v>360</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>18</v>
-      </c>
       <c r="H4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30">
       <c r="A5" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B5" s="3">
         <f>322</f>
@@ -1200,21 +1200,21 @@
         <v>150</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="4" t="s">
-        <v>21</v>
-      </c>
       <c r="H5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="60">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" s="3">
         <v>349</v>
@@ -1223,79 +1223,79 @@
         <v>250</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="4" t="s">
-        <v>25</v>
-      </c>
       <c r="H6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="90">
       <c r="A7" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3">
         <v>200</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="H7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30">
       <c r="A8" s="10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3">
         <v>100</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="H8" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30">
       <c r="A9" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="E9" s="11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H9" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="45">
       <c r="A10" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" s="3">
         <v>441</v>
@@ -1304,21 +1304,21 @@
         <v>150</v>
       </c>
       <c r="E10" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="G10" s="4" t="s">
-        <v>35</v>
-      </c>
       <c r="H10" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="45">
       <c r="A11" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B11" s="3">
         <v>500</v>
@@ -1327,21 +1327,21 @@
         <v>200</v>
       </c>
       <c r="E11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G11" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="H11" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="75">
       <c r="A12" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B12" s="3">
         <v>240</v>
@@ -1350,21 +1350,21 @@
         <v>90</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G12" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="4" t="s">
-        <v>42</v>
-      </c>
       <c r="H12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30">
       <c r="A13" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B13" s="3">
         <v>210</v>
@@ -1373,21 +1373,21 @@
         <v>100</v>
       </c>
       <c r="E13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="G13" s="4" t="s">
-        <v>45</v>
-      </c>
       <c r="H13" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="45">
       <c r="A14" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B14" s="3">
         <v>164</v>
@@ -1396,21 +1396,21 @@
         <v>60</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G14" s="4" t="s">
-        <v>49</v>
-      </c>
       <c r="H14" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="75">
       <c r="A15" s="10" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B15" s="3">
         <v>710</v>
@@ -1419,21 +1419,21 @@
         <v>100</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F15" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="G15" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="H15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30">
       <c r="A16" s="10" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B16" s="3">
         <v>100</v>
@@ -1442,42 +1442,42 @@
         <v>50</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F16" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="G16" s="4" t="s">
-        <v>53</v>
-      </c>
       <c r="H16" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="75">
       <c r="A17" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3">
         <v>50</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="F17" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="H17" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="75">
       <c r="A18" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B18" s="3">
         <v>150</v>
@@ -1486,21 +1486,21 @@
         <v>50</v>
       </c>
       <c r="E18" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>61</v>
-      </c>
       <c r="H18" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="10" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B19" s="3">
         <v>100</v>
@@ -1509,21 +1509,21 @@
         <v>40</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F19" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="G19" s="4" t="s">
-        <v>63</v>
-      </c>
       <c r="H19" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30">
       <c r="A20" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B20" s="3">
         <v>119</v>
@@ -1532,42 +1532,42 @@
         <v>40</v>
       </c>
       <c r="E20" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="G20" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="G20" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="H20" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="45">
       <c r="A21" s="10" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="3">
         <v>40</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="F21" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="H21" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30">
       <c r="A22" s="10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B22" s="3">
         <v>100</v>
@@ -1576,21 +1576,21 @@
         <v>40</v>
       </c>
       <c r="E22" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="G22" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="G22" s="6" t="s">
-        <v>73</v>
-      </c>
       <c r="H22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="75">
       <c r="A23" s="10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B23" s="3">
         <v>590</v>
@@ -1599,21 +1599,21 @@
         <v>75</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F23" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="G23" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="H23" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30">
       <c r="A24" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B24" s="3">
         <v>40</v>
@@ -1622,100 +1622,100 @@
         <v>30</v>
       </c>
       <c r="E24" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="G24" s="4" t="s">
-        <v>78</v>
-      </c>
       <c r="H24" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="45">
       <c r="A25" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3">
         <v>25</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G25" s="1"/>
       <c r="H25" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="45">
       <c r="A26" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="3">
         <v>20</v>
       </c>
       <c r="D26" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E26" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="H26" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="30">
       <c r="A27" s="10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3">
         <v>20</v>
       </c>
       <c r="E27" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="F27" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="H27" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="30">
       <c r="A28" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3">
         <v>20</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="F28" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F28" s="1" t="s">
-        <v>88</v>
-      </c>
       <c r="H28" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="60">
       <c r="A29" s="10" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B29" s="3">
         <v>40</v>
@@ -1724,21 +1724,21 @@
         <v>20</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F29" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G29" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G29" s="4" t="s">
-        <v>90</v>
-      </c>
       <c r="H29" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="30">
       <c r="A30" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B30" s="3">
         <v>299</v>
@@ -1747,21 +1747,21 @@
         <v>60</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F30" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G30" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="G30" s="8" t="s">
-        <v>93</v>
-      </c>
       <c r="H30" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B31" s="3">
         <v>35</v>
@@ -1770,21 +1770,21 @@
         <v>18</v>
       </c>
       <c r="E31" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G31" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="G31" s="4" t="s">
-        <v>97</v>
-      </c>
       <c r="H31" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B32" s="3">
         <v>50</v>
@@ -1793,21 +1793,21 @@
         <v>10</v>
       </c>
       <c r="E32" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F32" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="G32" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="G32" s="4" t="s">
-        <v>101</v>
-      </c>
       <c r="H32" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="30">
       <c r="A33" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B33" s="3">
         <v>30</v>
@@ -1816,37 +1816,37 @@
         <v>10</v>
       </c>
       <c r="E33" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="F33" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="H33" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="30">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="45">
       <c r="A34" s="10" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="3">
         <v>5</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G34" s="9"/>
       <c r="H34" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="10" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="3">
@@ -1854,35 +1854,35 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="30">
       <c r="A36" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="3">
         <v>10</v>
       </c>
       <c r="E36" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F36" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="G36" s="1"/>
       <c r="H36" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B37" s="3">
         <v>55</v>
@@ -1891,73 +1891,73 @@
         <v>20</v>
       </c>
       <c r="E37" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="G37" s="4" t="s">
-        <v>113</v>
-      </c>
       <c r="H37" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="3">
         <v>10</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H38" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B39" s="3"/>
       <c r="C39" s="3">
         <v>5</v>
       </c>
       <c r="E39" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F39" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F39" s="1" t="s">
-        <v>117</v>
-      </c>
       <c r="H39" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B40" s="3"/>
       <c r="C40" s="3">
         <v>5</v>
       </c>
       <c r="E40" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="F40" s="1" t="s">
-        <v>120</v>
-      </c>
       <c r="H40" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="41" spans="1:8">

</xml_diff>

<commit_message>
sold 12 items to CW
</commit_message>
<xml_diff>
--- a/files/selling_table.xlsx
+++ b/files/selling_table.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lgc2035/Documents/lawrence-chillrud.github.io/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B77F0D95-731A-054D-9DDB-1B42F6BCA762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06455159-336A-D14B-8B74-A3287B38AAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{2C9E99C7-C0A1-7B43-AFD4-86135AAC3BC4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="115">
   <si>
     <t>Item</t>
   </si>
@@ -81,12 +81,6 @@
   </si>
   <si>
     <t>Segata Light Oak 60" Media Console</t>
-  </si>
-  <si>
-    <t>ac</t>
-  </si>
-  <si>
-    <t>Midea 12,000 BTU Smart Inverter Window Air Conditioner with MShield</t>
   </si>
   <si>
     <t>Computer monitor (x2)</t>
@@ -167,18 +161,6 @@
     </r>
   </si>
   <si>
-    <t>IKEA Butcher Block</t>
-  </si>
-  <si>
-    <t>Bought in 2022. Heavy, good quality wood top. Some cosmetic scratches on surface</t>
-  </si>
-  <si>
-    <t>butcher_block</t>
-  </si>
-  <si>
-    <t>IKEA VADHOLMA Kitchen island, black/oak, 31 1/8x24 5/8x35 3/8 "</t>
-  </si>
-  <si>
     <t>Folding tatami mat - Queen</t>
   </si>
   <si>
@@ -195,27 +177,6 @@
   </si>
   <si>
     <t>Sorens 70.5" Pantry</t>
-  </si>
-  <si>
-    <t>Microwave</t>
-  </si>
-  <si>
-    <t>Regularly cleaned, works perfectly! Used to be one of Wirecutter's picks for best microwaves.</t>
-  </si>
-  <si>
-    <t>microwave</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="10"/>
-        <color rgb="FF1155CC"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>TOSHIBA EM131A5C-BS Countertop Microwave Ovens 1.2 Cu Ft, 12.4" Removable Turntable Smart Humidity Sensor 12 Auto Menus Mute Function ECO Mode Easy Clean Interior Black Color 1100W</t>
-    </r>
   </si>
   <si>
     <t>bed</t>
@@ -290,15 +251,6 @@
     </r>
   </si>
   <si>
-    <t>43.25x27.5x29.75</t>
-  </si>
-  <si>
-    <t>Great condition, some very minor surface pen marks that could be sanded out.</t>
-  </si>
-  <si>
-    <t>desk</t>
-  </si>
-  <si>
     <t>Easy to buy replacement filters, in great condition.</t>
   </si>
   <si>
@@ -326,48 +278,6 @@
     <t>wifi</t>
   </si>
   <si>
-    <t>Kitchen Table</t>
-  </si>
-  <si>
-    <t>44.75x27.5x29.25</t>
-  </si>
-  <si>
-    <t>kitchen_table</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comfortable, clean, soft seat with rolly wheels &amp; adjustable height. </t>
-  </si>
-  <si>
-    <t>chair_swivel</t>
-  </si>
-  <si>
-    <t>Tower fan</t>
-  </si>
-  <si>
-    <t>13x13x38</t>
-  </si>
-  <si>
-    <t>Works great! Multiple settings, speeds, oscillates, quiet, etc.</t>
-  </si>
-  <si>
-    <t>fan</t>
-  </si>
-  <si>
-    <t>knife_holder</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="10"/>
-        <color rgb="FF1155CC"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Modern Innovations 16 Inch Stainless Steel Magnetic Knife Bar - Use as Knife Holder, Knife Rack, Knife Strip, Kitchen Utensil Holder and Tool Holder</t>
-    </r>
-  </si>
-  <si>
     <t>Vacuum cleaner</t>
   </si>
   <si>
@@ -377,18 +287,6 @@
     <t>Shark Navigator Deluxe Upright Vacuum</t>
   </si>
   <si>
-    <t>Immersion blender</t>
-  </si>
-  <si>
-    <t>Bought in 2026, works great!</t>
-  </si>
-  <si>
-    <t>blender</t>
-  </si>
-  <si>
-    <t>Hamilton Beach 2-Speed Hand Blender with Whisk Attachment, New, 59762F</t>
-  </si>
-  <si>
     <t>Weber grill</t>
   </si>
   <si>
@@ -425,30 +323,6 @@
     <t>basket</t>
   </si>
   <si>
-    <t>Trashcan</t>
-  </si>
-  <si>
-    <t>Good condition.</t>
-  </si>
-  <si>
-    <t>trashcan</t>
-  </si>
-  <si>
-    <t>45L Rectangular Step Trash Can Silver - Brightroom™: Stainless Steel, Quiet Pedal Lid, Removable Liner, Kitchen Use</t>
-  </si>
-  <si>
-    <t>mop</t>
-  </si>
-  <si>
-    <t>Dish drying rack</t>
-  </si>
-  <si>
-    <t>Fits small surfaces perfectly.</t>
-  </si>
-  <si>
-    <t>drying_rack</t>
-  </si>
-  <si>
     <t>Utensil holders</t>
   </si>
   <si>
@@ -491,9 +365,6 @@
     <t>Space heater</t>
   </si>
   <si>
-    <t>Wooden desk</t>
-  </si>
-  <si>
     <t>Air purifier</t>
   </si>
   <si>
@@ -512,18 +383,6 @@
     <t>Xfinity Wifi Modem+Router Gateway (Xb6-t Xfi). Supports strong speeds, works great, no connectivity issues.</t>
   </si>
   <si>
-    <t>Classic kitchen table! Some marks from use but functions and still looks great.</t>
-  </si>
-  <si>
-    <t>Office chair</t>
-  </si>
-  <si>
-    <t>Magnetic knife holders (x2)</t>
-  </si>
-  <si>
-    <t>Holds kitchen knives/metal utensils perfectly, attaches with command strips. Selling the pair for $20 or individually for $15 each.</t>
-  </si>
-  <si>
     <t>Bought in 2022. Works great, filter cleaned regularly!</t>
   </si>
   <si>
@@ -566,22 +425,10 @@
     <t>So your veggies don't fall out on the grill! Genius. Clean and in great condition.</t>
   </si>
   <si>
-    <t>Bona mop, heads &amp; cleaner refills</t>
-  </si>
-  <si>
-    <t>Bona Premium Microfiber Floor Mop for Dry and Wet Floor Cleaning - Includes Microfiber Cleaning Pad and Microfiber Dusting Pad</t>
-  </si>
-  <si>
     <t>Article brand, bought new in 2022, in mint condition.</t>
   </si>
   <si>
     <t>Article TV stand/console</t>
-  </si>
-  <si>
-    <t>Bought at the start of summer 2026, in mint condition. Wirecutter's top pick for best AC! Super quiet and cools our apartment really well.</t>
-  </si>
-  <si>
-    <t>Midea AC – 12,000 BTU</t>
   </si>
 </sst>
 </file>
@@ -591,7 +438,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -637,14 +484,6 @@
       <name val="Var(--skin-header-font)"/>
     </font>
     <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -675,11 +514,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -700,14 +538,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -746,7 +582,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1FB07438-A594-274B-871C-20F9770322F7}" name="Table_2" displayName="Table_2" ref="A2:H41" headerRowCount="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1FB07438-A594-274B-871C-20F9770322F7}" name="Table_2" displayName="Table_2" ref="A2:H29" headerRowCount="0">
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{03249C9C-63FD-9B4A-A6FA-34F534EB3AA8}" name="Column1"/>
     <tableColumn id="2" xr3:uid="{249238A1-8479-7447-A9AC-A39DAD7BE156}" name="Column2"/>
@@ -1078,7 +914,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21BAEBAA-1347-2A45-BA72-46E5B69F16C0}">
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="32.33203125" bestFit="1" customWidth="1"/>
@@ -1112,7 +948,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>142</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="60">
@@ -1135,12 +971,12 @@
         <v>10</v>
       </c>
       <c r="H2" t="s">
-        <v>144</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="30">
       <c r="A3" s="10" t="s">
-        <v>157</v>
+        <v>114</v>
       </c>
       <c r="B3" s="3">
         <v>849</v>
@@ -1152,7 +988,7 @@
         <v>11</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>156</v>
+        <v>113</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>12</v>
@@ -1161,170 +997,170 @@
         <v>13</v>
       </c>
       <c r="H3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="60">
-      <c r="A4" s="10" t="s">
-        <v>159</v>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="B4" s="3">
-        <v>430</v>
-      </c>
-      <c r="C4" s="3">
-        <v>360</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="30">
-      <c r="A5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="3">
         <f>322</f>
         <v>322</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C4" s="3">
         <f>150</f>
         <v>150</v>
       </c>
-      <c r="E5" s="11" t="s">
-        <v>118</v>
+      <c r="E4" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="60">
+      <c r="A5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="3">
+        <v>349</v>
+      </c>
+      <c r="C5" s="3">
+        <v>250</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="60">
-      <c r="A6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="3">
-        <v>349</v>
-      </c>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="90">
+      <c r="A6" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="3"/>
       <c r="C6" s="3">
-        <v>250</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>20</v>
+        <v>200</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>84</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" s="4" t="s">
         <v>22</v>
       </c>
       <c r="H6" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="90">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="30">
       <c r="A7" s="10" t="s">
-        <v>119</v>
+        <v>85</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>120</v>
+        <v>86</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>24</v>
       </c>
       <c r="H7" t="s">
-        <v>144</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30">
-      <c r="A8" s="10" t="s">
-        <v>121</v>
+      <c r="A8" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="B8" s="3"/>
-      <c r="C8" s="3">
-        <v>100</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>25</v>
-      </c>
+      <c r="C8" s="3"/>
       <c r="E8" s="11" t="s">
-        <v>122</v>
+        <v>87</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>26</v>
       </c>
       <c r="H8" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="30">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="45">
       <c r="A9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
+      <c r="B9" s="3">
+        <v>441</v>
+      </c>
+      <c r="C9" s="3">
+        <v>150</v>
+      </c>
       <c r="E9" s="11" t="s">
-        <v>123</v>
+        <v>28</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>30</v>
       </c>
       <c r="H9" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="45">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="75">
       <c r="A10" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B10" s="3">
-        <v>441</v>
+        <v>240</v>
       </c>
       <c r="C10" s="3">
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>30</v>
+        <v>109</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H10" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="45">
-      <c r="A11" s="1" t="s">
-        <v>33</v>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="30">
+      <c r="A11" s="10" t="s">
+        <v>88</v>
       </c>
       <c r="B11" s="3">
-        <v>500</v>
+        <v>210</v>
       </c>
       <c r="C11" s="3">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>34</v>
@@ -1336,90 +1172,88 @@
         <v>36</v>
       </c>
       <c r="H11" t="s">
-        <v>148</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="75">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" s="3">
+        <v>710</v>
+      </c>
+      <c r="C12" s="3">
+        <v>100</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="3">
-        <v>240</v>
-      </c>
-      <c r="C12" s="3">
-        <v>90</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G12" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="H12" t="s">
-        <v>143</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30">
       <c r="A13" s="10" t="s">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="B13" s="3">
-        <v>210</v>
+        <v>100</v>
       </c>
       <c r="C13" s="3">
-        <v>100</v>
-      </c>
-      <c r="E13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="H13" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="75">
+      <c r="A14" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3">
+        <v>50</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="H13" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="45">
-      <c r="A14" s="1" t="s">
+      <c r="E14" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="3">
-        <v>164</v>
-      </c>
-      <c r="C14" s="3">
-        <v>60</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="H14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="75">
+      <c r="A15" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="B15" s="3">
+        <v>150</v>
+      </c>
+      <c r="C15" s="3">
+        <v>50</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="H14" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="75">
-      <c r="A15" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="B15" s="3">
-        <v>710</v>
-      </c>
-      <c r="C15" s="3">
-        <v>100</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>149</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>47</v>
@@ -1428,21 +1262,21 @@
         <v>48</v>
       </c>
       <c r="H15" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="30">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" s="10" t="s">
-        <v>126</v>
+        <v>92</v>
       </c>
       <c r="B16" s="3">
         <v>100</v>
       </c>
       <c r="C16" s="3">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>49</v>
@@ -1451,560 +1285,297 @@
         <v>50</v>
       </c>
       <c r="H16" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="75">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="30">
       <c r="A17" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3">
+        <v>119</v>
+      </c>
       <c r="C17" s="3">
-        <v>50</v>
-      </c>
-      <c r="D17" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="F17" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H17" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="75">
-      <c r="A18" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="30">
+      <c r="A18" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="3">
+        <v>100</v>
+      </c>
+      <c r="C18" s="3">
+        <v>40</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="3">
-        <v>150</v>
-      </c>
-      <c r="C18" s="3">
-        <v>50</v>
-      </c>
-      <c r="E18" s="2" t="s">
+      <c r="F18" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="H18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="75">
+      <c r="A19" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B19" s="3">
+        <v>590</v>
+      </c>
+      <c r="C19" s="3">
+        <v>75</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="H18" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="B19" s="3">
-        <v>100</v>
-      </c>
-      <c r="C19" s="3">
+      <c r="G19" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H19" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="30">
+      <c r="A20" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B20" s="3">
         <v>40</v>
       </c>
-      <c r="E19" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G19" s="4" t="s">
+      <c r="C20" s="3">
+        <v>30</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="H19" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="30">
-      <c r="A20" s="1" t="s">
+      <c r="F20" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B20" s="3">
-        <v>119</v>
-      </c>
-      <c r="C20" s="3">
-        <v>40</v>
-      </c>
-      <c r="E20" s="2" t="s">
+      <c r="G20" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>64</v>
-      </c>
       <c r="H20" t="s">
-        <v>148</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="45">
       <c r="A21" s="10" t="s">
-        <v>129</v>
+        <v>97</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="3">
-        <v>40</v>
-      </c>
-      <c r="D21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G21" s="1"/>
+      <c r="H21" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="30">
+      <c r="A22" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="3">
+        <v>299</v>
+      </c>
+      <c r="C22" s="3">
+        <v>60</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="G22" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="H22" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="H21" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="30">
-      <c r="A22" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="B22" s="3">
-        <v>100</v>
-      </c>
-      <c r="C22" s="3">
-        <v>40</v>
-      </c>
-      <c r="E22" s="2" t="s">
+      <c r="B23" s="3">
+        <v>50</v>
+      </c>
+      <c r="C23" s="3">
+        <v>10</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F23" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="G23" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="H22" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="75">
-      <c r="A23" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="B23" s="3">
-        <v>590</v>
-      </c>
-      <c r="C23" s="3">
-        <v>75</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="F23" s="1" t="s">
+      <c r="H23" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="30">
+      <c r="A24" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="B24" s="3">
+        <v>30</v>
+      </c>
+      <c r="C24" s="3">
+        <v>10</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H23" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="30">
-      <c r="A24" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="B24" s="3">
-        <v>40</v>
-      </c>
-      <c r="C24" s="3">
-        <v>30</v>
-      </c>
-      <c r="E24" s="2" t="s">
+      <c r="F24" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="H24" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="45">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="30">
       <c r="A25" s="10" t="s">
-        <v>134</v>
+        <v>111</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="G25" s="1"/>
+        <v>112</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="G25" s="9"/>
       <c r="H25" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="45">
-      <c r="A26" s="1" t="s">
-        <v>77</v>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="10" t="s">
+        <v>100</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="3">
-        <v>20</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>136</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E26" s="2"/>
       <c r="F26" s="1" t="s">
-        <v>79</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="G26" s="1"/>
       <c r="H26" t="s">
-        <v>148</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="30">
-      <c r="A27" s="10" t="s">
-        <v>137</v>
+      <c r="A27" s="1" t="s">
+        <v>76</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>81</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="G27" s="1"/>
       <c r="H27" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="30">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3">
-        <v>20</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>83</v>
+        <v>5</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H28" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="60">
-      <c r="A29" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="B29" s="3">
-        <v>40</v>
-      </c>
-      <c r="C29" s="3">
-        <v>20</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H29" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="30">
-      <c r="A30" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B30" s="3">
-        <v>299</v>
-      </c>
-      <c r="C30" s="3">
-        <v>60</v>
-      </c>
-      <c r="E30" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G30" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="H30" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8">
-      <c r="A31" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="B31" s="3">
-        <v>35</v>
-      </c>
-      <c r="C31" s="3">
-        <v>18</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G31" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="H31" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
-      <c r="A32" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B32" s="3">
-        <v>50</v>
-      </c>
-      <c r="C32" s="3">
-        <v>10</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="G32" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="H32" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="30">
-      <c r="A33" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="B33" s="3">
-        <v>30</v>
-      </c>
-      <c r="C33" s="3">
-        <v>10</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="H33" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="45">
-      <c r="A34" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3">
-        <v>5</v>
-      </c>
-      <c r="E34" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="G34" s="9"/>
-      <c r="H34" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
-      <c r="A35" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3">
-        <v>10</v>
-      </c>
-      <c r="E35" s="2"/>
-      <c r="F35" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="G35" s="1"/>
-      <c r="H35" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="30">
-      <c r="A36" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3">
-        <v>10</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G36" s="1"/>
-      <c r="H36" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
-      <c r="A37" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B37" s="3">
-        <v>55</v>
-      </c>
-      <c r="C37" s="3">
-        <v>20</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="G37" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="H37" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
-      <c r="A38" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3">
-        <v>10</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G38" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="H38" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
-      <c r="A39" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3">
-        <v>5</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="H39" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
-      <c r="A40" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3">
-        <v>5</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="H40" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
-      <c r="A41" s="1"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="1"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="1"/>
-    </row>
-    <row r="42" spans="1:8">
-      <c r="A42" s="1"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="1"/>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" s="1"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="1"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="G3" r:id="rId1" xr:uid="{54A10D3A-39CF-3742-B73D-0564A216F4C6}"/>
-    <hyperlink ref="G4" r:id="rId2" xr:uid="{94D08A13-7D4F-A347-B335-65C2E5DE7E83}"/>
-    <hyperlink ref="G5" r:id="rId3" xr:uid="{02AEAE82-B705-164E-A34D-505F6F672D0D}"/>
-    <hyperlink ref="G6" r:id="rId4" xr:uid="{E0E930FE-9BD4-3B47-9801-8B8BDB0F00AC}"/>
-    <hyperlink ref="G10" r:id="rId5" xr:uid="{E116A338-9CC6-7A4E-81E0-1280822D2BD4}"/>
-    <hyperlink ref="G11" r:id="rId6" xr:uid="{975F3BAC-708D-FF4C-9F6E-0C67B93D26CF}"/>
-    <hyperlink ref="G12" r:id="rId7" xr:uid="{7B99AF8A-4346-5C4B-A1E9-FB7ECF3D1818}"/>
-    <hyperlink ref="G13" r:id="rId8" xr:uid="{74691A7C-3D4E-5A49-ADFD-94751FAEB8A2}"/>
-    <hyperlink ref="G14" r:id="rId9" xr:uid="{802C3451-19C3-C141-A7ED-6172DAAE38FB}"/>
-    <hyperlink ref="G15" r:id="rId10" xr:uid="{19D2F7B9-9EC6-A54D-B987-512645DA8431}"/>
-    <hyperlink ref="G16" r:id="rId11" xr:uid="{23967684-D66E-404C-B5CA-BBB0D3BDA0C4}"/>
-    <hyperlink ref="G18" r:id="rId12" xr:uid="{7ABBF447-72DA-5745-9F7C-A8F38949FB97}"/>
-    <hyperlink ref="G19" r:id="rId13" xr:uid="{3CF4353A-DABA-E746-B86C-052CD57FCAF0}"/>
-    <hyperlink ref="G20" r:id="rId14" xr:uid="{534386FD-F962-D74D-AFB3-3209792E9AF4}"/>
-    <hyperlink ref="G22" r:id="rId15" xr:uid="{7BF600C8-12B5-5440-A21D-840ED35F7F7B}"/>
-    <hyperlink ref="G23" r:id="rId16" xr:uid="{D94A8EFA-F618-4447-82E2-8AC7245F52E6}"/>
-    <hyperlink ref="G24" r:id="rId17" xr:uid="{D7A8E1F2-EE7D-5F4E-820A-F48A5F13DC4A}"/>
-    <hyperlink ref="G29" r:id="rId18" xr:uid="{D0BAFFD0-DBE4-DC4E-ACF9-759E2E07C8E9}"/>
-    <hyperlink ref="G30" r:id="rId19" xr:uid="{F234B5D1-13C0-1646-AD21-D683B24B1A57}"/>
-    <hyperlink ref="G31" r:id="rId20" xr:uid="{84822F22-48D3-C145-86C6-28DFFA148BE6}"/>
-    <hyperlink ref="G32" r:id="rId21" xr:uid="{7CFD0808-E22E-4D41-8646-08108D857A6C}"/>
-    <hyperlink ref="G37" r:id="rId22" xr:uid="{421D543C-3547-BA45-BA9E-C377A9FE6983}"/>
-    <hyperlink ref="G38" r:id="rId23" xr:uid="{F4D6804E-3E12-6345-8647-A104700BD757}"/>
+    <hyperlink ref="G4" r:id="rId2" xr:uid="{02AEAE82-B705-164E-A34D-505F6F672D0D}"/>
+    <hyperlink ref="G5" r:id="rId3" xr:uid="{E0E930FE-9BD4-3B47-9801-8B8BDB0F00AC}"/>
+    <hyperlink ref="G9" r:id="rId4" xr:uid="{E116A338-9CC6-7A4E-81E0-1280822D2BD4}"/>
+    <hyperlink ref="G10" r:id="rId5" xr:uid="{7B99AF8A-4346-5C4B-A1E9-FB7ECF3D1818}"/>
+    <hyperlink ref="G11" r:id="rId6" xr:uid="{74691A7C-3D4E-5A49-ADFD-94751FAEB8A2}"/>
+    <hyperlink ref="G12" r:id="rId7" xr:uid="{19D2F7B9-9EC6-A54D-B987-512645DA8431}"/>
+    <hyperlink ref="G13" r:id="rId8" xr:uid="{23967684-D66E-404C-B5CA-BBB0D3BDA0C4}"/>
+    <hyperlink ref="G15" r:id="rId9" xr:uid="{7ABBF447-72DA-5745-9F7C-A8F38949FB97}"/>
+    <hyperlink ref="G16" r:id="rId10" xr:uid="{3CF4353A-DABA-E746-B86C-052CD57FCAF0}"/>
+    <hyperlink ref="G17" r:id="rId11" xr:uid="{534386FD-F962-D74D-AFB3-3209792E9AF4}"/>
+    <hyperlink ref="G18" r:id="rId12" xr:uid="{7BF600C8-12B5-5440-A21D-840ED35F7F7B}"/>
+    <hyperlink ref="G19" r:id="rId13" xr:uid="{D94A8EFA-F618-4447-82E2-8AC7245F52E6}"/>
+    <hyperlink ref="G20" r:id="rId14" xr:uid="{D7A8E1F2-EE7D-5F4E-820A-F48A5F13DC4A}"/>
+    <hyperlink ref="G22" r:id="rId15" xr:uid="{F234B5D1-13C0-1646-AD21-D683B24B1A57}"/>
+    <hyperlink ref="G23" r:id="rId16" xr:uid="{7CFD0808-E22E-4D41-8646-08108D857A6C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId24"/>
+    <tablePart r:id="rId17"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
removed avs purchases from listings
</commit_message>
<xml_diff>
--- a/files/selling_table.xlsx
+++ b/files/selling_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lgc2035/Documents/lawrence-chillrud.github.io/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06455159-336A-D14B-8B74-A3287B38AAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{301A5F4A-4A65-BC41-B9BD-2B1FB69B9A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{2C9E99C7-C0A1-7B43-AFD4-86135AAC3BC4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="103">
   <si>
     <t>Item</t>
   </si>
@@ -170,15 +170,6 @@
     <t>Folding Tatami Mat</t>
   </si>
   <si>
-    <t>Bought in 2022, in great condition, offers tons of pantry storage.</t>
-  </si>
-  <si>
-    <t>kitchen_hutch</t>
-  </si>
-  <si>
-    <t>Sorens 70.5" Pantry</t>
-  </si>
-  <si>
     <t>bed</t>
   </si>
   <si>
@@ -230,36 +221,6 @@
     <t>perfect aire 1500/900/600W 7-Fin 25" Oil-Filled Radiator Heater, White</t>
   </si>
   <si>
-    <t>Toaster oven</t>
-  </si>
-  <si>
-    <t>Wirecutter's pick for the best small toaster oven! Works perfectly.</t>
-  </si>
-  <si>
-    <t>toaster</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="10"/>
-        <color rgb="FF1155CC"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Panasonic FlashXpress Compact Toaster Oven with Double Infrared Heating, Crumb Tray and 1300 Watts of Cooking Power - 4 Slice Countertop Toaster Oven - NB-G110P (Stainless Steel)</t>
-    </r>
-  </si>
-  <si>
-    <t>Easy to buy replacement filters, in great condition.</t>
-  </si>
-  <si>
-    <t>air_purifier</t>
-  </si>
-  <si>
-    <t>Levoit Core® 300-P Air Purifier</t>
-  </si>
-  <si>
     <t>tatami_queen</t>
   </si>
   <si>
@@ -350,9 +311,6 @@
     <t>TBD. Will take pictures of which plants we're selling in August!</t>
   </si>
   <si>
-    <t>Kitchen hutch/pantry</t>
-  </si>
-  <si>
     <t>Queen futon bed</t>
   </si>
   <si>
@@ -363,9 +321,6 @@
   </si>
   <si>
     <t>Space heater</t>
-  </si>
-  <si>
-    <t>Air purifier</t>
   </si>
   <si>
     <t>Floor tatami mats  - Queen (x2)</t>
@@ -438,7 +393,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -463,12 +418,6 @@
       <u/>
       <sz val="10"/>
       <color rgb="FF1155CC"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -517,7 +466,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -528,18 +477,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -582,7 +525,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1FB07438-A594-274B-871C-20F9770322F7}" name="Table_2" displayName="Table_2" ref="A2:H29" headerRowCount="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1FB07438-A594-274B-871C-20F9770322F7}" name="Table_2" displayName="Table_2" ref="A2:H26" headerRowCount="0">
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{03249C9C-63FD-9B4A-A6FA-34F534EB3AA8}" name="Column1"/>
     <tableColumn id="2" xr3:uid="{249238A1-8479-7447-A9AC-A39DAD7BE156}" name="Column2"/>
@@ -914,7 +857,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21BAEBAA-1347-2A45-BA72-46E5B69F16C0}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="32.33203125" bestFit="1" customWidth="1"/>
@@ -948,7 +891,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="60">
@@ -971,12 +914,12 @@
         <v>10</v>
       </c>
       <c r="H2" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="30">
-      <c r="A3" s="10" t="s">
-        <v>114</v>
+      <c r="A3" s="8" t="s">
+        <v>102</v>
       </c>
       <c r="B3" s="3">
         <v>849</v>
@@ -987,8 +930,8 @@
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="11" t="s">
-        <v>113</v>
+      <c r="E3" s="9" t="s">
+        <v>101</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>12</v>
@@ -997,7 +940,7 @@
         <v>13</v>
       </c>
       <c r="H3" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30">
@@ -1012,8 +955,8 @@
         <f>150</f>
         <v>150</v>
       </c>
-      <c r="E4" s="11" t="s">
-        <v>82</v>
+      <c r="E4" s="9" t="s">
+        <v>72</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>15</v>
@@ -1022,7 +965,7 @@
         <v>16</v>
       </c>
       <c r="H4" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="60">
@@ -1045,12 +988,12 @@
         <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="90">
-      <c r="A6" s="10" t="s">
-        <v>83</v>
+      <c r="A6" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3">
@@ -1059,19 +1002,19 @@
       <c r="D6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>84</v>
+      <c r="E6" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H6" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30">
-      <c r="A7" s="10" t="s">
-        <v>85</v>
+      <c r="A7" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3">
@@ -1080,14 +1023,14 @@
       <c r="D7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="11" t="s">
-        <v>86</v>
+      <c r="E7" s="9" t="s">
+        <v>76</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>24</v>
       </c>
       <c r="H7" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30">
@@ -1096,14 +1039,14 @@
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
-      <c r="E8" s="11" t="s">
-        <v>87</v>
+      <c r="E8" s="9" t="s">
+        <v>77</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>26</v>
       </c>
       <c r="H8" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="45">
@@ -1116,7 +1059,7 @@
       <c r="C9" s="3">
         <v>150</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="9" t="s">
         <v>28</v>
       </c>
       <c r="F9" s="1" t="s">
@@ -1126,7 +1069,7 @@
         <v>30</v>
       </c>
       <c r="H9" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="75">
@@ -1139,8 +1082,8 @@
       <c r="C10" s="3">
         <v>90</v>
       </c>
-      <c r="E10" s="11" t="s">
-        <v>109</v>
+      <c r="E10" s="9" t="s">
+        <v>97</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>32</v>
@@ -1149,409 +1092,340 @@
         <v>33</v>
       </c>
       <c r="H10" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="30">
-      <c r="A11" s="10" t="s">
-        <v>88</v>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="75">
+      <c r="A11" s="8" t="s">
+        <v>78</v>
       </c>
       <c r="B11" s="3">
-        <v>210</v>
+        <v>710</v>
       </c>
       <c r="C11" s="3">
         <v>100</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="H11" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="30">
+      <c r="A12" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="3">
+        <v>100</v>
+      </c>
+      <c r="C12" s="3">
+        <v>50</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H11" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="75">
-      <c r="A12" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="B12" s="3">
-        <v>710</v>
-      </c>
-      <c r="C12" s="3">
-        <v>100</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="H12" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="75">
+      <c r="A13" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H12" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="30">
-      <c r="A13" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B13" s="3">
-        <v>100</v>
-      </c>
+      <c r="B13" s="3"/>
       <c r="C13" s="3">
         <v>50</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="D13" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" t="s">
         <v>91</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H13" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="75">
       <c r="A14" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="3"/>
+        <v>42</v>
+      </c>
+      <c r="B14" s="3">
+        <v>150</v>
+      </c>
       <c r="C14" s="3">
         <v>50</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="E14" s="2" t="s">
         <v>43</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>44</v>
       </c>
+      <c r="G14" s="4" t="s">
+        <v>45</v>
+      </c>
       <c r="H14" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="75">
-      <c r="A15" s="1" t="s">
-        <v>45</v>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="8" t="s">
+        <v>81</v>
       </c>
       <c r="B15" s="3">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="C15" s="3">
+        <v>40</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H15" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="75">
+      <c r="A16" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="3">
+        <v>590</v>
+      </c>
+      <c r="C16" s="3">
+        <v>75</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="H16" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="30">
+      <c r="A17" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="3">
+        <v>40</v>
+      </c>
+      <c r="C17" s="3">
+        <v>30</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H15" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" s="10" t="s">
+      <c r="F17" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H17" t="s">
         <v>92</v>
       </c>
-      <c r="B16" s="3">
-        <v>100</v>
-      </c>
-      <c r="C16" s="3">
-        <v>40</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G16" s="4" t="s">
+    </row>
+    <row r="18" spans="1:8" ht="45">
+      <c r="A18" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3">
+        <v>25</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G18" s="1"/>
+      <c r="H18" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="30">
+      <c r="A19" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="3">
+        <v>299</v>
+      </c>
+      <c r="C19" s="3">
+        <v>60</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H19" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B20" s="3">
         <v>50</v>
       </c>
-      <c r="H16" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="30">
-      <c r="A17" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B17" s="3">
-        <v>119</v>
-      </c>
-      <c r="C17" s="3">
-        <v>40</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="H17" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="30">
-      <c r="A18" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="B18" s="3">
-        <v>100</v>
-      </c>
-      <c r="C18" s="3">
-        <v>40</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H18" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="75">
-      <c r="A19" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B19" s="3">
-        <v>590</v>
-      </c>
-      <c r="C19" s="3">
-        <v>75</v>
-      </c>
-      <c r="E19" s="11" t="s">
+      <c r="C20" s="3">
+        <v>10</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H20" t="s">
         <v>95</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="H19" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="30">
-      <c r="A20" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B20" s="3">
-        <v>40</v>
-      </c>
-      <c r="C20" s="3">
+    </row>
+    <row r="21" spans="1:8" ht="30">
+      <c r="A21" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="3">
         <v>30</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G20" s="4" t="s">
+      <c r="C21" s="3">
+        <v>10</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="H20" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="45">
-      <c r="A21" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3">
-        <v>25</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>98</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G21" s="1"/>
       <c r="H21" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3">
+        <v>5</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="3">
-        <v>299</v>
-      </c>
-      <c r="C22" s="3">
-        <v>60</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>66</v>
-      </c>
+      <c r="G22" s="7"/>
       <c r="H22" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B23" s="3">
-        <v>50</v>
-      </c>
+      <c r="A23" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="3"/>
       <c r="C23" s="3">
         <v>10</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>68</v>
-      </c>
+      <c r="E23" s="2"/>
       <c r="F23" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>70</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="G23" s="1"/>
       <c r="H23" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30">
       <c r="A24" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B24" s="3">
-        <v>30</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="B24" s="3"/>
       <c r="C24" s="3">
         <v>10</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>73</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="G24" s="1"/>
       <c r="H24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="30">
-      <c r="A25" s="10" t="s">
-        <v>111</v>
+        <v>94</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3">
         <v>5</v>
       </c>
-      <c r="E25" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="G25" s="9"/>
+      <c r="E25" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="H25" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="10" t="s">
-        <v>100</v>
-      </c>
+      <c r="A26" s="1"/>
       <c r="B26" s="3"/>
-      <c r="C26" s="3">
-        <v>10</v>
-      </c>
+      <c r="C26" s="3"/>
+      <c r="D26" s="1"/>
       <c r="E26" s="2"/>
-      <c r="F26" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="G26" s="1"/>
-      <c r="H26" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="30">
-      <c r="A27" s="1" t="s">
-        <v>76</v>
-      </c>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="1"/>
       <c r="B27" s="3"/>
-      <c r="C27" s="3">
-        <v>10</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="G27" s="1"/>
-      <c r="H27" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
-      <c r="A28" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3">
-        <v>5</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H28" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
-      <c r="A29" s="1"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="1"/>
-    </row>
-    <row r="30" spans="1:8">
-      <c r="A30" s="1"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="1"/>
+      <c r="C27" s="3"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1560,22 +1434,19 @@
     <hyperlink ref="G5" r:id="rId3" xr:uid="{E0E930FE-9BD4-3B47-9801-8B8BDB0F00AC}"/>
     <hyperlink ref="G9" r:id="rId4" xr:uid="{E116A338-9CC6-7A4E-81E0-1280822D2BD4}"/>
     <hyperlink ref="G10" r:id="rId5" xr:uid="{7B99AF8A-4346-5C4B-A1E9-FB7ECF3D1818}"/>
-    <hyperlink ref="G11" r:id="rId6" xr:uid="{74691A7C-3D4E-5A49-ADFD-94751FAEB8A2}"/>
-    <hyperlink ref="G12" r:id="rId7" xr:uid="{19D2F7B9-9EC6-A54D-B987-512645DA8431}"/>
-    <hyperlink ref="G13" r:id="rId8" xr:uid="{23967684-D66E-404C-B5CA-BBB0D3BDA0C4}"/>
-    <hyperlink ref="G15" r:id="rId9" xr:uid="{7ABBF447-72DA-5745-9F7C-A8F38949FB97}"/>
-    <hyperlink ref="G16" r:id="rId10" xr:uid="{3CF4353A-DABA-E746-B86C-052CD57FCAF0}"/>
-    <hyperlink ref="G17" r:id="rId11" xr:uid="{534386FD-F962-D74D-AFB3-3209792E9AF4}"/>
-    <hyperlink ref="G18" r:id="rId12" xr:uid="{7BF600C8-12B5-5440-A21D-840ED35F7F7B}"/>
-    <hyperlink ref="G19" r:id="rId13" xr:uid="{D94A8EFA-F618-4447-82E2-8AC7245F52E6}"/>
-    <hyperlink ref="G20" r:id="rId14" xr:uid="{D7A8E1F2-EE7D-5F4E-820A-F48A5F13DC4A}"/>
-    <hyperlink ref="G22" r:id="rId15" xr:uid="{F234B5D1-13C0-1646-AD21-D683B24B1A57}"/>
-    <hyperlink ref="G23" r:id="rId16" xr:uid="{7CFD0808-E22E-4D41-8646-08108D857A6C}"/>
+    <hyperlink ref="G11" r:id="rId6" xr:uid="{19D2F7B9-9EC6-A54D-B987-512645DA8431}"/>
+    <hyperlink ref="G12" r:id="rId7" xr:uid="{23967684-D66E-404C-B5CA-BBB0D3BDA0C4}"/>
+    <hyperlink ref="G14" r:id="rId8" xr:uid="{7ABBF447-72DA-5745-9F7C-A8F38949FB97}"/>
+    <hyperlink ref="G15" r:id="rId9" xr:uid="{3CF4353A-DABA-E746-B86C-052CD57FCAF0}"/>
+    <hyperlink ref="G16" r:id="rId10" xr:uid="{D94A8EFA-F618-4447-82E2-8AC7245F52E6}"/>
+    <hyperlink ref="G17" r:id="rId11" xr:uid="{D7A8E1F2-EE7D-5F4E-820A-F48A5F13DC4A}"/>
+    <hyperlink ref="G19" r:id="rId12" xr:uid="{F234B5D1-13C0-1646-AD21-D683B24B1A57}"/>
+    <hyperlink ref="G20" r:id="rId13" xr:uid="{7CFD0808-E22E-4D41-8646-08108D857A6C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId17"/>
+    <tablePart r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>